<commit_message>
Improve Excel form layout for efficient manual entry
- Color-coded rows: sections, steps, auto-filled vs manual input
- Yellow input cells and mark column for checkboxes/ratings
- Header legend, frozen panes, data validation for ✓/✗ and 1-5
- Add LAYOUT_EXAMPLE.txt guide in download folder

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/download/TEST_Checklist.xlsx
+++ b/equipment-templates/output/download/TEST_Checklist.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Checklist'!$1:$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,105 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE699"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +133,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4B4B4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -411,664 +561,650 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="56" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Поле</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Отметка</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Отметка ✓/✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Жёлтые ячейки — ввод вручную  |  Голубые — из базы  |  Колонка «Отметка» — ✓ / ✗ / 1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>ЧЕК-ЛИСТ БАЗОВОЙ ПРОВЕРКИ АППАРАТА (5-7 минут)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>БЛОК А. РЕКВИЗИТЫ АППАРАТА (для дальнейшего анализа)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Модель</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Kyocera ECOSYS M3040dn</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr"/>
+      <c r="D5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Серийный номер</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>LS67Y43279</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr"/>
+      <c r="D6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Инвентарный номер</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>67+</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr"/>
+      <c r="D7" s="9" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Локация (офис/кабинет)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Риелторы (Тюмень)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr"/>
+      <c r="D8" s="9" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Модель картриджа</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="8" t="inlineStr"/>
+      <c r="D9" s="9" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Текущий ресурс картриджа (%)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr"/>
+      <c r="C10" s="8" t="inlineStr"/>
+      <c r="D10" s="9" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Дата последнего ТО</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr"/>
+      <c r="C11" s="8" t="inlineStr"/>
+      <c r="D11" s="9" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Дата последней замены ЗИП</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr"/>
+      <c r="C12" s="8" t="inlineStr"/>
+      <c r="D12" s="9" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Ответственный у Заказчика</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr"/>
+      <c r="C13" s="8" t="inlineStr"/>
+      <c r="D13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Контакт (тел/email)</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
+      <c r="D14" s="9" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>БЛОК Б. ПРОВЕРКА ПО ШАГАМ</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>ШАГ 1. ВНЕШНИЙ ОСМОТР (30 сек)</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Корпус, крышки, лотки — визуально целые</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr"/>
+      <c r="C17" s="8" t="inlineStr"/>
+      <c r="D17" s="15" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Кабели подключены надежно, без перегибов</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr"/>
+      <c r="C18" s="8" t="inlineStr"/>
+      <c r="D18" s="15" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Вокруг аппарата чисто, нет мусора, скрепок, скоб</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr"/>
+      <c r="C19" s="8" t="inlineStr"/>
+      <c r="D19" s="15" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>ШАГ 2. СЧЕТЧИКИ (1 мин)</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>Открыть меню → Отчет → Страница состояния (Kyocera)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr"/>
+      <c r="C21" s="8" t="inlineStr"/>
+      <c r="D21" s="15" t="inlineStr"/>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>или Меню → Reports → Usage Report (HP)</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
         <is>
           <t>Записать: Total / ЧБ / Цвет / Сканер</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr"/>
+      <c r="C23" s="8" t="inlineStr"/>
+      <c r="D23" s="15" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="13" t="inlineStr">
         <is>
           <t>Сверить с данными в файле "Этажи покопийка AI.xlsx"</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr"/>
+      <c r="C24" s="8" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>(расхождение &gt; 5% — пометить в карточке)</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>ШАГ 3. ТЕСТОВАЯ ПЕЧАТЬ (1 мин)</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Распечатать тестовую страницу из встроенного меню</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr"/>
+      <c r="C27" s="8" t="inlineStr"/>
+      <c r="D27" s="15" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="13" t="inlineStr">
         <is>
           <t>Оценить: плотность, полосы, фон, регистрация</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr"/>
+      <c r="C28" s="8" t="inlineStr"/>
+      <c r="D28" s="15" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Проверить закрепление тонера (провести пальцем)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr"/>
+      <c r="C29" s="8" t="inlineStr"/>
+      <c r="D29" s="15" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Для цветных — напечатать страницу качества цвета</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr"/>
+      <c r="C30" s="8" t="inlineStr"/>
+      <c r="D30" s="15" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t>ШАГ 4. ТЕСТ СКАНИРОВАНИЯ (1 мин)</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
         <is>
           <t>Положить лист A4 на стекло / в ADF</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr"/>
+      <c r="C32" s="8" t="inlineStr"/>
+      <c r="D32" s="15" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
         <is>
           <t>Отсканировать на email / в сетевую папку</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr"/>
+      <c r="C33" s="8" t="inlineStr"/>
+      <c r="D33" s="15" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="13" t="inlineStr">
         <is>
           <t>Проверить: нет полос, захват ADF без перекоса</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr"/>
+      <c r="C34" s="8" t="inlineStr"/>
+      <c r="D34" s="15" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t>ШАГ 5. ФИЗИКА (1-2 мин)</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
         <is>
           <t>Открыть переднюю крышку, заглянуть внутрь</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr"/>
+      <c r="C36" s="8" t="inlineStr"/>
+      <c r="D36" s="15" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>Осмотреть ролики захвата (лысые? грязные?)</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr"/>
+      <c r="C37" s="8" t="inlineStr"/>
+      <c r="D37" s="15" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Осмотреть термоузел (следы тонера, нагар?)</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="B38" s="14" t="inlineStr"/>
+      <c r="C38" s="8" t="inlineStr"/>
+      <c r="D38" s="15" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>Проверить дуплекс (нет ли замятой бумаги)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr"/>
+      <c r="C39" s="8" t="inlineStr"/>
+      <c r="D39" s="15" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>Понюхать (запах гари = проблема с печкой)</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="B40" s="14" t="inlineStr"/>
+      <c r="C40" s="8" t="inlineStr"/>
+      <c r="D40" s="15" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t>ШАГ 6. СУБЪЕКТИВНАЯ ОЦЕНКА (30 сек)</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Оценить физическое состояние (1-5)</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="B42" s="14" t="inlineStr"/>
+      <c r="C42" s="8" t="inlineStr"/>
+      <c r="D42" s="15" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Оценить качество печати (1-5)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="B43" s="14" t="inlineStr"/>
+      <c r="C43" s="8" t="inlineStr"/>
+      <c r="D43" s="15" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>Оценить качество сканирования (1-5)</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="B44" s="14" t="inlineStr"/>
+      <c r="C44" s="8" t="inlineStr"/>
+      <c r="D44" s="15" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>Выставить общую оценку (1-5)</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="B45" s="14" t="inlineStr"/>
+      <c r="C45" s="8" t="inlineStr"/>
+      <c r="D45" s="15" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t>ШАГ 7. ФИКСАЦИЯ В КАРТОЧКЕ</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Заполнить все поля карточки аппарата</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="B47" s="14" t="inlineStr"/>
+      <c r="C47" s="8" t="inlineStr"/>
+      <c r="D47" s="15" t="inlineStr"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>Отметить все применимые пункты "План действий"</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="B48" s="14" t="inlineStr"/>
+      <c r="C48" s="8" t="inlineStr"/>
+      <c r="D48" s="15" t="inlineStr"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>Указать приоритет и срок выполнения</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="B49" s="14" t="inlineStr"/>
+      <c r="C49" s="8" t="inlineStr"/>
+      <c r="D49" s="15" t="inlineStr"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Сфотографировать дефекты (если есть)</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
-      <c r="D49" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="B50" s="14" t="inlineStr"/>
+      <c r="C50" s="8" t="inlineStr"/>
+      <c r="D50" s="15" t="inlineStr"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
         <is>
           <t>🚨 КРАСНЫЕ ФЛАГИ (немедленная эскалация Наталье, руководителю)</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
-      <c r="D50" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="B51" s="10" t="inlineStr"/>
+      <c r="C51" s="8" t="inlineStr"/>
+      <c r="D51" s="9" t="inlineStr"/>
+    </row>
+    <row r="52" ht="28" customHeight="1">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>• Аппарат не включается / нет реакции</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
-      <c r="D51" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr"/>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>• Счетчик не изменился с прошлого месяца (0 отпечатков)</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
-      <c r="C52" t="inlineStr"/>
-      <c r="D52" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="B53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54" ht="28" customHeight="1">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>• Сильный запах гари, дым</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
-      <c r="D53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr"/>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>• Треск, скрежет, посторонние звуки</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
-      <c r="D54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56" ht="28" customHeight="1">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>• Явное физическое повреждение корпуса/лотков</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr"/>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>• Оценка "1" по любому из параметров</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58" ht="28" customHeight="1">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>• Аппарат отсутствует на месте (пропажа / перемещение без согласования)</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
-      <c r="D57" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="B58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>• Конфликт с Заказчиком / отказ в доступе</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
-      <c r="D58" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="B59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60" ht="28" customHeight="1">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>• Риск срыва SLA (критичный фронт-офис не работает)</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
-      <c r="D59" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr"/>
+    </row>
+    <row r="61" ht="20" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
         <is>
           <t>Канал эскалации</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" s="7" t="inlineStr">
         <is>
           <t>мессенджер MAX → чат "Этажи_Сервис"</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr"/>
-      <c r="D60" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="C61" s="8" t="inlineStr"/>
+      <c r="D61" s="9" t="inlineStr"/>
+    </row>
+    <row r="62" ht="20" customHeight="1">
+      <c r="A62" s="6" t="inlineStr">
         <is>
           <t>Время реакции Натальи</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B62" s="7" t="inlineStr">
         <is>
           <t>до 30 минут в рабочее время</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr"/>
-      <c r="D61" t="inlineStr"/>
+      <c r="C62" s="8" t="inlineStr"/>
+      <c r="D62" s="9" t="inlineStr"/>
     </row>
   </sheetData>
+  <mergeCells count="22">
+    <mergeCell ref="B60:D60"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B59:D59"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="B58:D58"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="D17 D18 D19 D21 D23 D24 D27 D28 D29 D30 D32 D33 D34 D36 D37 D38 D39 D40 D42 D43 D44 D45 D47 D48 D49 D50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"✓,✗,—"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Layout v3: numbered field form wins over compact (716 vs 378)
- Compare 2 layouts on Kyocera + HP Color device profiles
- Winner: field layout with № column, device strip, section gaps
- Fix Ед./№ columns broken by pandas itertuples
- Dropdown lists for marks, alert styling for red flags
- Add layout_review.py and compare samples in download/compare/

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/download/TEST_Checklist.xlsx
+++ b/equipment-templates/output/download/TEST_Checklist.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,16 +42,22 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
@@ -86,6 +92,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
@@ -116,16 +127,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFE699"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -147,11 +153,39 @@
         <color rgb="00B4B4B4"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="00BF8F00"/>
+      </left>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top style="medium">
+        <color rgb="00BF8F00"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C65911"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C65911"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C65911"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C65911"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -160,42 +194,45 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -563,32 +600,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Поле</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Значение</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Ед.</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Отметка ✓/✗</t>
         </is>
@@ -597,610 +640,773 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Жёлтые ячейки — ввод вручную  |  Голубые — из базы  |  Колонка «Отметка» — ✓ / ✗ / 1-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="28" customHeight="1">
+          <t>№ = пункт проверки  |  Жёлтые = ввод  |  Голубые = из базы  |  Отметка: ✓ / ✗ / 1-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>ЧЕК-ЛИСТ БАЗОВОЙ ПРОВЕРКИ АППАРАТА (5-7 минут)</t>
+          <t>Модель: Kyocera ECOSYS M3040dn  |  Серийный: LS67Y43279  |  Инв. 67+  |  Локация: Риелторы (Тюмень)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
+          <t>ЧЕК-ЛИСТ БАЗОВОЙ ПРОВЕРКИ АППАРАТА (5-7 минут)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="5" t="inlineStr"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
           <t>БЛОК А. РЕКВИЗИТЫ АППАРАТА (для дальнейшего анализа)</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Модель</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Kyocera ECOSYS M3040dn</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr"/>
-      <c r="D5" s="9" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr"/>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr"/>
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Серийный номер</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>LS67Y43279</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr"/>
-      <c r="D6" s="9" t="inlineStr"/>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr"/>
+      <c r="E7" s="11" t="inlineStr"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Инвентарный номер</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>67+</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr"/>
-      <c r="D7" s="9" t="inlineStr"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr"/>
+      <c r="E8" s="11" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr"/>
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Локация (офис/кабинет)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>Риелторы (Тюмень)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr"/>
-      <c r="D8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr"/>
+      <c r="E9" s="11" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Модель картриджа</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="8" t="inlineStr"/>
-      <c r="D9" s="9" t="inlineStr"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
+      <c r="C10" s="12" t="inlineStr"/>
+      <c r="D10" s="10" t="inlineStr"/>
+      <c r="E10" s="11" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr"/>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Текущий ресурс картриджа (%)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr"/>
-      <c r="C10" s="8" t="inlineStr"/>
-      <c r="D10" s="9" t="inlineStr"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr"/>
+      <c r="D11" s="10" t="inlineStr"/>
+      <c r="E11" s="11" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Дата последнего ТО</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr"/>
-      <c r="C11" s="8" t="inlineStr"/>
-      <c r="D11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="C12" s="12" t="inlineStr"/>
+      <c r="D12" s="10" t="inlineStr"/>
+      <c r="E12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="5" t="inlineStr"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Дата последней замены ЗИП</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr"/>
-      <c r="C12" s="8" t="inlineStr"/>
-      <c r="D12" s="9" t="inlineStr"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr"/>
+      <c r="D13" s="10" t="inlineStr"/>
+      <c r="E13" s="11" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Ответственный у Заказчика</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr"/>
-      <c r="C13" s="8" t="inlineStr"/>
-      <c r="D13" s="9" t="inlineStr"/>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr"/>
+      <c r="D14" s="10" t="inlineStr"/>
+      <c r="E14" s="11" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="5" t="inlineStr"/>
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Контакт (тел/email)</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr"/>
-      <c r="C14" s="8" t="inlineStr"/>
-      <c r="D14" s="9" t="inlineStr"/>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="11" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="13" t="inlineStr">
         <is>
           <t>БЛОК Б. ПРОВЕРКА ПО ШАГАМ</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="12" t="inlineStr">
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>ШАГ 1. ВНЕШНИЙ ОСМОТР (30 сек)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="13" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Корпус, крышки, лотки — визуально целые</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="8" t="inlineStr"/>
-      <c r="D17" s="15" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr"/>
+      <c r="D18" s="10" t="inlineStr"/>
+      <c r="E18" s="16" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Кабели подключены надежно, без перегибов</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr"/>
-      <c r="C18" s="8" t="inlineStr"/>
-      <c r="D18" s="15" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr"/>
+      <c r="D19" s="10" t="inlineStr"/>
+      <c r="E19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Вокруг аппарата чисто, нет мусора, скрепок, скоб</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr"/>
-      <c r="C19" s="8" t="inlineStr"/>
-      <c r="D19" s="15" t="inlineStr"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr"/>
+      <c r="D20" s="10" t="inlineStr"/>
+      <c r="E20" s="16" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>ШАГ 2. СЧЕТЧИКИ (1 мин)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="13" t="inlineStr">
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Открыть меню → Отчет → Страница состояния (Kyocera)</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr"/>
-      <c r="C21" s="8" t="inlineStr"/>
-      <c r="D21" s="15" t="inlineStr"/>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr"/>
+      <c r="D22" s="10" t="inlineStr"/>
+      <c r="E22" s="16" t="inlineStr"/>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="5" t="inlineStr"/>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>или Меню → Reports → Usage Report (HP)</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>Записать: Total / ЧБ / Цвет / Сканер</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr"/>
-      <c r="C23" s="8" t="inlineStr"/>
-      <c r="D23" s="15" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr"/>
+      <c r="D24" s="10" t="inlineStr"/>
+      <c r="E24" s="16" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Сверить с данными в файле "Этажи покопийка AI.xlsx"</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr"/>
-      <c r="C24" s="8" t="inlineStr"/>
-      <c r="D24" s="15" t="inlineStr"/>
-    </row>
-    <row r="25" ht="28" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr"/>
+      <c r="D25" s="10" t="inlineStr"/>
+      <c r="E25" s="16" t="inlineStr"/>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="A26" s="5" t="inlineStr"/>
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>(расхождение &gt; 5% — пометить в карточке)</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>ШАГ 3. ТЕСТОВАЯ ПЕЧАТЬ (1 мин)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
         <is>
           <t>Распечатать тестовую страницу из встроенного меню</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr"/>
-      <c r="C27" s="8" t="inlineStr"/>
-      <c r="D27" s="15" t="inlineStr"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr"/>
+      <c r="D28" s="10" t="inlineStr"/>
+      <c r="E28" s="16" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
         <is>
           <t>Оценить: плотность, полосы, фон, регистрация</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr"/>
-      <c r="C28" s="8" t="inlineStr"/>
-      <c r="D28" s="15" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr"/>
+      <c r="D29" s="10" t="inlineStr"/>
+      <c r="E29" s="16" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Проверить закрепление тонера (провести пальцем)</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr"/>
-      <c r="C29" s="8" t="inlineStr"/>
-      <c r="D29" s="15" t="inlineStr"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr"/>
+      <c r="D30" s="10" t="inlineStr"/>
+      <c r="E30" s="16" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
         <is>
           <t>Для цветных — напечатать страницу качества цвета</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr"/>
-      <c r="C30" s="8" t="inlineStr"/>
-      <c r="D30" s="15" t="inlineStr"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr"/>
+      <c r="D31" s="10" t="inlineStr"/>
+      <c r="E31" s="16" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="14" t="inlineStr">
         <is>
           <t>ШАГ 4. ТЕСТ СКАНИРОВАНИЯ (1 мин)</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="13" t="inlineStr">
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
         <is>
           <t>Положить лист A4 на стекло / в ADF</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr"/>
-      <c r="C32" s="8" t="inlineStr"/>
-      <c r="D32" s="15" t="inlineStr"/>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="C33" s="15" t="inlineStr"/>
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="16" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t>Отсканировать на email / в сетевую папку</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr"/>
-      <c r="C33" s="8" t="inlineStr"/>
-      <c r="D33" s="15" t="inlineStr"/>
-    </row>
-    <row r="34" ht="20" customHeight="1">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="C34" s="15" t="inlineStr"/>
+      <c r="D34" s="10" t="inlineStr"/>
+      <c r="E34" s="16" t="inlineStr"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>Проверить: нет полос, захват ADF без перекоса</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr"/>
-      <c r="C34" s="8" t="inlineStr"/>
-      <c r="D34" s="15" t="inlineStr"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="C35" s="15" t="inlineStr"/>
+      <c r="D35" s="10" t="inlineStr"/>
+      <c r="E35" s="16" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>ШАГ 5. ФИЗИКА (1-2 мин)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="13" t="inlineStr">
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
         <is>
           <t>Открыть переднюю крышку, заглянуть внутрь</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr"/>
-      <c r="C36" s="8" t="inlineStr"/>
-      <c r="D36" s="15" t="inlineStr"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr"/>
+      <c r="D37" s="10" t="inlineStr"/>
+      <c r="E37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>Осмотреть ролики захвата (лысые? грязные?)</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr"/>
-      <c r="C37" s="8" t="inlineStr"/>
-      <c r="D37" s="15" t="inlineStr"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr"/>
+      <c r="D38" s="10" t="inlineStr"/>
+      <c r="E38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
         <is>
           <t>Осмотреть термоузел (следы тонера, нагар?)</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr"/>
-      <c r="C38" s="8" t="inlineStr"/>
-      <c r="D38" s="15" t="inlineStr"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr"/>
+      <c r="D39" s="10" t="inlineStr"/>
+      <c r="E39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>Проверить дуплекс (нет ли замятой бумаги)</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr"/>
-      <c r="C39" s="8" t="inlineStr"/>
-      <c r="D39" s="15" t="inlineStr"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="C40" s="15" t="inlineStr"/>
+      <c r="D40" s="10" t="inlineStr"/>
+      <c r="E40" s="16" t="inlineStr"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Понюхать (запах гари = проблема с печкой)</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr"/>
-      <c r="C40" s="8" t="inlineStr"/>
-      <c r="D40" s="15" t="inlineStr"/>
-    </row>
-    <row r="41" ht="20" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr"/>
+      <c r="D41" s="10" t="inlineStr"/>
+      <c r="E41" s="16" t="inlineStr"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>ШАГ 6. СУБЪЕКТИВНАЯ ОЦЕНКА (30 сек)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
         <is>
           <t>Оценить физическое состояние (1-5)</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr"/>
-      <c r="C42" s="8" t="inlineStr"/>
-      <c r="D42" s="15" t="inlineStr"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr"/>
+      <c r="D43" s="10" t="inlineStr"/>
+      <c r="E43" s="16" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Оценить качество печати (1-5)</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr"/>
-      <c r="C43" s="8" t="inlineStr"/>
-      <c r="D43" s="15" t="inlineStr"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="13" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr"/>
+      <c r="D44" s="10" t="inlineStr"/>
+      <c r="E44" s="16" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
         <is>
           <t>Оценить качество сканирования (1-5)</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr"/>
-      <c r="C44" s="8" t="inlineStr"/>
-      <c r="D44" s="15" t="inlineStr"/>
-    </row>
-    <row r="45" ht="20" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr"/>
+      <c r="D45" s="10" t="inlineStr"/>
+      <c r="E45" s="16" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
         <is>
           <t>Выставить общую оценку (1-5)</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr"/>
-      <c r="C45" s="8" t="inlineStr"/>
-      <c r="D45" s="15" t="inlineStr"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
-      <c r="A46" s="12" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr"/>
+      <c r="D46" s="10" t="inlineStr"/>
+      <c r="E46" s="16" t="inlineStr"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="14" t="inlineStr">
         <is>
           <t>ШАГ 7. ФИКСАЦИЯ В КАРТОЧКЕ</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="20" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
         <is>
           <t>Заполнить все поля карточки аппарата</t>
         </is>
       </c>
-      <c r="B47" s="14" t="inlineStr"/>
-      <c r="C47" s="8" t="inlineStr"/>
-      <c r="D47" s="15" t="inlineStr"/>
-    </row>
-    <row r="48" ht="20" customHeight="1">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="C48" s="15" t="inlineStr"/>
+      <c r="D48" s="10" t="inlineStr"/>
+      <c r="E48" s="16" t="inlineStr"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
         <is>
           <t>Отметить все применимые пункты "План действий"</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr"/>
-      <c r="C48" s="8" t="inlineStr"/>
-      <c r="D48" s="15" t="inlineStr"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr"/>
+      <c r="D49" s="10" t="inlineStr"/>
+      <c r="E49" s="16" t="inlineStr"/>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
         <is>
           <t>Указать приоритет и срок выполнения</t>
         </is>
       </c>
-      <c r="B49" s="14" t="inlineStr"/>
-      <c r="C49" s="8" t="inlineStr"/>
-      <c r="D49" s="15" t="inlineStr"/>
-    </row>
-    <row r="50" ht="20" customHeight="1">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr"/>
+      <c r="D50" s="10" t="inlineStr"/>
+      <c r="E50" s="16" t="inlineStr"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
         <is>
           <t>Сфотографировать дефекты (если есть)</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr"/>
-      <c r="C50" s="8" t="inlineStr"/>
-      <c r="D50" s="15" t="inlineStr"/>
-    </row>
-    <row r="51" ht="20" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr"/>
+      <c r="D51" s="10" t="inlineStr"/>
+      <c r="E51" s="16" t="inlineStr"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>🚨 КРАСНЫЕ ФЛАГИ (немедленная эскалация Наталье, руководителю)</t>
         </is>
       </c>
-      <c r="B51" s="10" t="inlineStr"/>
-      <c r="C51" s="8" t="inlineStr"/>
-      <c r="D51" s="9" t="inlineStr"/>
-    </row>
-    <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="C52" s="12" t="inlineStr"/>
+      <c r="D52" s="10" t="inlineStr"/>
+      <c r="E52" s="11" t="inlineStr"/>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="5" t="inlineStr"/>
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>• Аппарат не включается / нет реакции</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr"/>
-    </row>
-    <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="C53" s="7" t="inlineStr"/>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="5" t="inlineStr"/>
+      <c r="B54" s="6" t="inlineStr">
         <is>
           <t>• Счетчик не изменился с прошлого месяца (0 отпечатков)</t>
         </is>
       </c>
-      <c r="B53" s="5" t="inlineStr"/>
-    </row>
-    <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="C54" s="7" t="inlineStr"/>
+    </row>
+    <row r="55" ht="32" customHeight="1">
+      <c r="A55" s="5" t="inlineStr"/>
+      <c r="B55" s="6" t="inlineStr">
         <is>
           <t>• Сильный запах гари, дым</t>
         </is>
       </c>
-      <c r="B54" s="5" t="inlineStr"/>
-    </row>
-    <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="C55" s="7" t="inlineStr"/>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>• Треск, скрежет, посторонние звуки</t>
         </is>
       </c>
-      <c r="B55" s="5" t="inlineStr"/>
-    </row>
-    <row r="56" ht="28" customHeight="1">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="C56" s="7" t="inlineStr"/>
+    </row>
+    <row r="57" ht="32" customHeight="1">
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>• Явное физическое повреждение корпуса/лотков</t>
         </is>
       </c>
-      <c r="B56" s="5" t="inlineStr"/>
-    </row>
-    <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="4" t="inlineStr">
+      <c r="C57" s="7" t="inlineStr"/>
+    </row>
+    <row r="58" ht="32" customHeight="1">
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>• Оценка "1" по любому из параметров</t>
         </is>
       </c>
-      <c r="B57" s="5" t="inlineStr"/>
-    </row>
-    <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="C58" s="7" t="inlineStr"/>
+    </row>
+    <row r="59" ht="32" customHeight="1">
+      <c r="A59" s="5" t="inlineStr"/>
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>• Аппарат отсутствует на месте (пропажа / перемещение без согласования)</t>
         </is>
       </c>
-      <c r="B58" s="5" t="inlineStr"/>
-    </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="C59" s="7" t="inlineStr"/>
+    </row>
+    <row r="60" ht="32" customHeight="1">
+      <c r="A60" s="5" t="inlineStr"/>
+      <c r="B60" s="6" t="inlineStr">
         <is>
           <t>• Конфликт с Заказчиком / отказ в доступе</t>
         </is>
       </c>
-      <c r="B59" s="5" t="inlineStr"/>
-    </row>
-    <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="C60" s="7" t="inlineStr"/>
+    </row>
+    <row r="61" ht="32" customHeight="1">
+      <c r="A61" s="5" t="inlineStr"/>
+      <c r="B61" s="6" t="inlineStr">
         <is>
           <t>• Риск срыва SLA (критичный фронт-офис не работает)</t>
         </is>
       </c>
-      <c r="B60" s="5" t="inlineStr"/>
-    </row>
-    <row r="61" ht="20" customHeight="1">
-      <c r="A61" s="6" t="inlineStr">
+      <c r="C61" s="7" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="8" t="inlineStr">
         <is>
           <t>Канал эскалации</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>мессенджер MAX → чат "Этажи_Сервис"</t>
         </is>
       </c>
-      <c r="C61" s="8" t="inlineStr"/>
-      <c r="D61" s="9" t="inlineStr"/>
-    </row>
-    <row r="62" ht="20" customHeight="1">
-      <c r="A62" s="6" t="inlineStr">
+      <c r="D62" s="10" t="inlineStr"/>
+      <c r="E62" s="11" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="5" t="inlineStr"/>
+      <c r="B63" s="8" t="inlineStr">
         <is>
           <t>Время реакции Натальи</t>
         </is>
       </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="C63" s="9" t="inlineStr">
         <is>
           <t>до 30 минут в рабочее время</t>
         </is>
       </c>
-      <c r="C62" s="8" t="inlineStr"/>
-      <c r="D62" s="9" t="inlineStr"/>
+      <c r="D63" s="10" t="inlineStr"/>
+      <c r="E63" s="11" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="A35:D35"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="A20:D20"/>
-    <mergeCell ref="B53:D53"/>
-    <mergeCell ref="A31:D31"/>
-    <mergeCell ref="A15:D15"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="A41:D41"/>
-    <mergeCell ref="A16:D16"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="A46:D46"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="B59:D59"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="B56:D56"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B52:D52"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="23">
+    <mergeCell ref="C54:E54"/>
+    <mergeCell ref="C55:E55"/>
+    <mergeCell ref="C56:E56"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="C60:E60"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C61:E61"/>
+    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="C57:E57"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="C53:E53"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A47:E47"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="C58:E58"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C26:E26"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D17 D18 D19 D21 D23 D24 D27 D28 D29 D30 D32 D33 D34 D36 D37 D38 D39 D40 D42 D43 D44 D45 D47 D48 D49 D50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E18 E19 E20 E22 E24 E25 E28 E29 E30 E31 E33 E34 E35 E37 E38 E39 E40 E41 E43 E44 E45 E46 E48 E49 E50 E51" showDropDown="1" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓,✗,—"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>